<commit_message>
feat: read suppliers and invoices from the lab API
- ReadConfig.xaml reads Data/Config.xlsx once into a dictionary
- GetFinanceData.xaml logs in with the Windows credential P02_LabApi
  (role finance), checks status and role, and reads all pages of
  /v1/suppliers and /v1/invoices into two data tables
- Config gets the new setting LabApiCredential
- RuleConfig.json sets ST-SEC-009 to Warning for this project, because
  the API needs the password as plain text in the JSON login body
- Test_GetFinanceData.xaml checks counts and two known records
- Packages: WebAPI 2.5.2, Credentials 3.1.1, UIAutomation 26.10.2
</commit_message>
<xml_diff>
--- a/P02-Finance-Invoice-Intake/Data/Config.xlsx
+++ b/P02-Finance-Invoice-Intake/Data/Config.xlsx
@@ -154,7 +154,13 @@
     <x:t>P01_HospitalDemo</x:t>
   </x:si>
   <x:si>
-    <x:t>Name of the Windows credential with the lab login (the password is not stored here)</x:t>
+    <x:t>LabApiCredential</x:t>
+  </x:si>
+  <x:si>
+    <x:t>P02_LabApi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name of the Windows credential with the lab API login, role finance (the password is not stored here)</x:t>
   </x:si>
   <x:si>
     <x:t>AttachmentFolder</x:t>
@@ -167,6 +173,9 @@
   </x:si>
   <x:si>
     <x:t>ReportFolder</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name of the Windows credential with the Personalportalen login (the password is not stored here)</x:t>
   </x:si>
   <x:si>
     <x:t>Output</x:t>
@@ -699,29 +708,40 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:3">
       <x:c r="A17" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B17" s="0" t="s">
+      <x:c r="C17" s="0" t="s">
         <x:v>48</x:v>
-      </x:c>
-      <x:c r="C17" s="0" t="s">
-        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:3">
       <x:c r="A18" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B18" s="0" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B18" s="0" t="s">
+      <x:c r="C18" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="C18" s="0" t="s">
+    </x:row>
+    <x:row r="19" spans="1:3">
+      <x:c r="A19" s="0" t="s">
         <x:v>52</x:v>
+      </x:c>
+      <x:c r="B19" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C19" s="0" t="s">
+        <x:v>55</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>